<commit_message>
Update Ventes-Stock PCT 2024-2026 (courbes).xlsx
</commit_message>
<xml_diff>
--- a/Ventes-Stock PCT 2024-2026 (courbes).xlsx
+++ b/Ventes-Stock PCT 2024-2026 (courbes).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ilhem\Desktop\LOGEXPERT\BIOCON\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B2F773C-30E0-4685-B3F6-3ED226F7DAF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7031304B-56A3-4FAF-9AEC-EFD1A62FE171}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{02106002-8DC5-4A0A-8EFA-7A1E47A939C5}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{02106002-8DC5-4A0A-8EFA-7A1E47A939C5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -693,6 +693,9 @@
                 <c:pt idx="26">
                   <c:v>1369</c:v>
                 </c:pt>
+                <c:pt idx="27">
+                  <c:v>658</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -1056,6 +1059,9 @@
                 <c:pt idx="26">
                   <c:v>987</c:v>
                 </c:pt>
+                <c:pt idx="27">
+                  <c:v>856</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -1419,6 +1425,9 @@
                 <c:pt idx="26">
                   <c:v>436</c:v>
                 </c:pt>
+                <c:pt idx="27">
+                  <c:v>311</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -1782,6 +1791,9 @@
                 <c:pt idx="26">
                   <c:v>1335</c:v>
                 </c:pt>
+                <c:pt idx="27">
+                  <c:v>922</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -2145,6 +2157,9 @@
                 <c:pt idx="26">
                   <c:v>1483</c:v>
                 </c:pt>
+                <c:pt idx="27">
+                  <c:v>1700</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -2506,6 +2521,9 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="26">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="27">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -2876,6 +2894,9 @@
                 </c:pt>
                 <c:pt idx="26">
                   <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>17</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3517,6 +3538,9 @@
                 <c:pt idx="26">
                   <c:v>3424</c:v>
                 </c:pt>
+                <c:pt idx="27">
+                  <c:v>5166</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -3868,6 +3892,9 @@
                 <c:pt idx="26">
                   <c:v>3998</c:v>
                 </c:pt>
+                <c:pt idx="27">
+                  <c:v>3142</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -4219,6 +4246,9 @@
                 <c:pt idx="26">
                   <c:v>13611</c:v>
                 </c:pt>
+                <c:pt idx="27">
+                  <c:v>13300</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -4570,6 +4600,9 @@
                 <c:pt idx="26">
                   <c:v>4682</c:v>
                 </c:pt>
+                <c:pt idx="27">
+                  <c:v>3760</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -4921,6 +4954,9 @@
                 <c:pt idx="26">
                   <c:v>13106</c:v>
                 </c:pt>
+                <c:pt idx="27">
+                  <c:v>11406</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -5270,6 +5306,9 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="26">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="27">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -5624,6 +5663,9 @@
                 </c:pt>
                 <c:pt idx="26">
                   <c:v>1994</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>1977</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -10534,6 +10576,27 @@
       <c r="C31" s="3" t="s">
         <v>26</v>
       </c>
+      <c r="D31" s="3">
+        <v>658</v>
+      </c>
+      <c r="E31" s="3">
+        <v>856</v>
+      </c>
+      <c r="F31" s="3">
+        <v>311</v>
+      </c>
+      <c r="G31" s="3">
+        <v>922</v>
+      </c>
+      <c r="H31" s="3">
+        <v>1700</v>
+      </c>
+      <c r="I31" s="3">
+        <v>0</v>
+      </c>
+      <c r="J31" s="3">
+        <v>17</v>
+      </c>
     </row>
     <row r="32" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B32" s="4">
@@ -11463,6 +11526,27 @@
       <c r="C31" s="3" t="s">
         <v>26</v>
       </c>
+      <c r="D31" s="3">
+        <v>5166</v>
+      </c>
+      <c r="E31" s="3">
+        <v>3142</v>
+      </c>
+      <c r="F31" s="3">
+        <v>13300</v>
+      </c>
+      <c r="G31" s="3">
+        <v>3760</v>
+      </c>
+      <c r="H31" s="3">
+        <v>11406</v>
+      </c>
+      <c r="I31" s="3">
+        <v>0</v>
+      </c>
+      <c r="J31" s="3">
+        <v>1977</v>
+      </c>
     </row>
     <row r="32" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B32" s="4">

</xml_diff>

<commit_message>
chore: Mettre a jour les donnees de stock et de ventes PCT 2024-2026
</commit_message>
<xml_diff>
--- a/Ventes-Stock PCT 2024-2026 (courbes).xlsx
+++ b/Ventes-Stock PCT 2024-2026 (courbes).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ilhem\Desktop\LOGEXPERT\BIOCON\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7031304B-56A3-4FAF-9AEC-EFD1A62FE171}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F27F549E-FC6E-48EF-8275-68C529C56439}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{02106002-8DC5-4A0A-8EFA-7A1E47A939C5}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{02106002-8DC5-4A0A-8EFA-7A1E47A939C5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -696,6 +696,9 @@
                 <c:pt idx="27">
                   <c:v>658</c:v>
                 </c:pt>
+                <c:pt idx="28">
+                  <c:v>799</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -1062,6 +1065,9 @@
                 <c:pt idx="27">
                   <c:v>856</c:v>
                 </c:pt>
+                <c:pt idx="28">
+                  <c:v>821</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -1428,6 +1434,9 @@
                 <c:pt idx="27">
                   <c:v>311</c:v>
                 </c:pt>
+                <c:pt idx="28">
+                  <c:v>151</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -1794,6 +1803,9 @@
                 <c:pt idx="27">
                   <c:v>922</c:v>
                 </c:pt>
+                <c:pt idx="28">
+                  <c:v>1136</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -2160,6 +2172,9 @@
                 <c:pt idx="27">
                   <c:v>1700</c:v>
                 </c:pt>
+                <c:pt idx="28">
+                  <c:v>1373</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -2524,6 +2539,9 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="27">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="28">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -2897,6 +2915,9 @@
                 </c:pt>
                 <c:pt idx="27">
                   <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>24</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3541,6 +3562,9 @@
                 <c:pt idx="27">
                   <c:v>5166</c:v>
                 </c:pt>
+                <c:pt idx="28">
+                  <c:v>4367</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -3895,6 +3919,9 @@
                 <c:pt idx="27">
                   <c:v>3142</c:v>
                 </c:pt>
+                <c:pt idx="28">
+                  <c:v>2321</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -4249,6 +4276,9 @@
                 <c:pt idx="27">
                   <c:v>13300</c:v>
                 </c:pt>
+                <c:pt idx="28">
+                  <c:v>13149</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -4603,6 +4633,9 @@
                 <c:pt idx="27">
                   <c:v>3760</c:v>
                 </c:pt>
+                <c:pt idx="28">
+                  <c:v>2624</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -4957,6 +4990,9 @@
                 <c:pt idx="27">
                   <c:v>11406</c:v>
                 </c:pt>
+                <c:pt idx="28">
+                  <c:v>10033</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -5309,6 +5345,9 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="27">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="28">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -5666,6 +5705,9 @@
                 </c:pt>
                 <c:pt idx="27">
                   <c:v>1977</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>1953</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -10605,6 +10647,27 @@
       <c r="C32" s="3" t="s">
         <v>13</v>
       </c>
+      <c r="D32" s="3">
+        <v>799</v>
+      </c>
+      <c r="E32" s="3">
+        <v>821</v>
+      </c>
+      <c r="F32" s="3">
+        <v>151</v>
+      </c>
+      <c r="G32" s="3">
+        <v>1136</v>
+      </c>
+      <c r="H32" s="3">
+        <v>1373</v>
+      </c>
+      <c r="I32" s="3">
+        <v>0</v>
+      </c>
+      <c r="J32" s="3">
+        <v>24</v>
+      </c>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B33" s="4">
@@ -11555,6 +11618,27 @@
       <c r="C32" s="3" t="s">
         <v>13</v>
       </c>
+      <c r="D32" s="3">
+        <v>4367</v>
+      </c>
+      <c r="E32" s="3">
+        <v>2321</v>
+      </c>
+      <c r="F32" s="3">
+        <v>13149</v>
+      </c>
+      <c r="G32" s="3">
+        <v>2624</v>
+      </c>
+      <c r="H32" s="3">
+        <v>10033</v>
+      </c>
+      <c r="I32" s="3">
+        <v>0</v>
+      </c>
+      <c r="J32" s="3">
+        <v>1953</v>
+      </c>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B33" s="4">

</xml_diff>